<commit_message>
Added NBA Results for Oct 20, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Times New Roman"/>
@@ -537,6 +535,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>113</v>
+      </c>
+      <c r="I2" t="n">
+        <v>121</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -570,6 +577,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>121</v>
+      </c>
+      <c r="I3" t="n">
+        <v>113</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -603,6 +619,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>106</v>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -636,6 +661,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" t="n">
+        <v>106</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -669,6 +703,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>116</v>
+      </c>
+      <c r="I6" t="n">
+        <v>104</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -701,6 +744,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H7" t="n">
+        <v>104</v>
+      </c>
+      <c r="I7" t="n">
+        <v>116</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Added NBA Results for Oct 22, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -1710,6 +1710,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H30" t="n">
+        <v>106</v>
+      </c>
+      <c r="I30" t="n">
+        <v>114</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1743,6 +1752,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H31" t="n">
+        <v>114</v>
+      </c>
+      <c r="I31" t="n">
+        <v>106</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1776,6 +1794,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H32" t="n">
+        <v>84</v>
+      </c>
+      <c r="I32" t="n">
+        <v>96</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1808,6 +1835,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H33" t="n">
+        <v>96</v>
+      </c>
+      <c r="I33" t="n">
+        <v>84</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Added NBA Results for Oct 23, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -1878,6 +1878,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H34" t="n">
+        <v>112</v>
+      </c>
+      <c r="I34" t="n">
+        <v>102</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1911,6 +1920,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H35" t="n">
+        <v>102</v>
+      </c>
+      <c r="I35" t="n">
+        <v>112</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1944,6 +1962,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H36" t="n">
+        <v>115</v>
+      </c>
+      <c r="I36" t="n">
+        <v>93</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -1977,6 +2004,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H37" t="n">
+        <v>93</v>
+      </c>
+      <c r="I37" t="n">
+        <v>115</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -2010,6 +2046,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H38" t="n">
+        <v>121</v>
+      </c>
+      <c r="I38" t="n">
+        <v>105</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -2043,6 +2088,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H39" t="n">
+        <v>105</v>
+      </c>
+      <c r="I39" t="n">
+        <v>121</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2076,6 +2130,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H40" t="n">
+        <v>128</v>
+      </c>
+      <c r="I40" t="n">
+        <v>81</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -2109,6 +2172,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H41" t="n">
+        <v>81</v>
+      </c>
+      <c r="I41" t="n">
+        <v>128</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -2142,6 +2214,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H42" t="n">
+        <v>103</v>
+      </c>
+      <c r="I42" t="n">
+        <v>107</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -2175,6 +2256,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H43" t="n">
+        <v>107</v>
+      </c>
+      <c r="I43" t="n">
+        <v>103</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -2208,6 +2298,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H44" t="n">
+        <v>128</v>
+      </c>
+      <c r="I44" t="n">
+        <v>111</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -2241,6 +2340,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H45" t="n">
+        <v>111</v>
+      </c>
+      <c r="I45" t="n">
+        <v>128</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -2274,6 +2382,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H46" t="n">
+        <v>132</v>
+      </c>
+      <c r="I46" t="n">
+        <v>125</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -2307,6 +2424,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H47" t="n">
+        <v>125</v>
+      </c>
+      <c r="I47" t="n">
+        <v>132</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -2340,6 +2466,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H48" t="n">
+        <v>114</v>
+      </c>
+      <c r="I48" t="n">
+        <v>110</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -2373,6 +2508,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H49" t="n">
+        <v>110</v>
+      </c>
+      <c r="I49" t="n">
+        <v>114</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -2406,6 +2550,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H50" t="n">
+        <v>119</v>
+      </c>
+      <c r="I50" t="n">
+        <v>120</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -2439,6 +2592,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H51" t="n">
+        <v>120</v>
+      </c>
+      <c r="I51" t="n">
+        <v>119</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -2472,6 +2634,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H52" t="n">
+        <v>117</v>
+      </c>
+      <c r="I52" t="n">
+        <v>125</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -2505,6 +2676,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H53" t="n">
+        <v>125</v>
+      </c>
+      <c r="I53" t="n">
+        <v>117</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -2538,6 +2718,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H54" t="n">
+        <v>128</v>
+      </c>
+      <c r="I54" t="n">
+        <v>120</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -2571,6 +2760,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H55" t="n">
+        <v>120</v>
+      </c>
+      <c r="I55" t="n">
+        <v>128</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -2604,6 +2802,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H56" t="n">
+        <v>111</v>
+      </c>
+      <c r="I56" t="n">
+        <v>108</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -2636,6 +2843,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H57" t="n">
+        <v>108</v>
+      </c>
+      <c r="I57" t="n">
+        <v>111</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
Added NBA Results for Oct 24, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -2886,6 +2886,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H58" t="n">
+        <v>110</v>
+      </c>
+      <c r="I58" t="n">
+        <v>115</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -2919,6 +2928,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H59" t="n">
+        <v>115</v>
+      </c>
+      <c r="I59" t="n">
+        <v>110</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -2952,6 +2970,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H60" t="n">
+        <v>116</v>
+      </c>
+      <c r="I60" t="n">
+        <v>127</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -2985,6 +3012,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H61" t="n">
+        <v>127</v>
+      </c>
+      <c r="I61" t="n">
+        <v>116</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3018,6 +3054,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H62" t="n">
+        <v>121</v>
+      </c>
+      <c r="I62" t="n">
+        <v>125</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -3051,6 +3096,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H63" t="n">
+        <v>125</v>
+      </c>
+      <c r="I63" t="n">
+        <v>121</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -3084,6 +3138,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H64" t="n">
+        <v>122</v>
+      </c>
+      <c r="I64" t="n">
+        <v>106</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -3117,6 +3180,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H65" t="n">
+        <v>106</v>
+      </c>
+      <c r="I65" t="n">
+        <v>122</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -3150,6 +3222,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H66" t="n">
+        <v>124</v>
+      </c>
+      <c r="I66" t="n">
+        <v>120</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -3183,6 +3264,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H67" t="n">
+        <v>120</v>
+      </c>
+      <c r="I67" t="n">
+        <v>124</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -3216,6 +3306,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H68" t="n">
+        <v>121</v>
+      </c>
+      <c r="I68" t="n">
+        <v>114</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -3249,6 +3348,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H69" t="n">
+        <v>114</v>
+      </c>
+      <c r="I69" t="n">
+        <v>121</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -3282,6 +3390,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H70" t="n">
+        <v>135</v>
+      </c>
+      <c r="I70" t="n">
+        <v>141</v>
+      </c>
+      <c r="J70" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -3315,6 +3432,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H71" t="n">
+        <v>141</v>
+      </c>
+      <c r="I71" t="n">
+        <v>135</v>
+      </c>
+      <c r="J71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -3348,6 +3474,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H72" t="n">
+        <v>122</v>
+      </c>
+      <c r="I72" t="n">
+        <v>131</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -3380,6 +3515,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H73" t="n">
+        <v>131</v>
+      </c>
+      <c r="I73" t="n">
+        <v>122</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
Added NBA Results for Oct 25, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -3558,6 +3558,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H74" t="n">
+        <v>132</v>
+      </c>
+      <c r="I74" t="n">
+        <v>123</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -3591,6 +3600,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H75" t="n">
+        <v>123</v>
+      </c>
+      <c r="I75" t="n">
+        <v>132</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -3624,6 +3642,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H76" t="n">
+        <v>136</v>
+      </c>
+      <c r="I76" t="n">
+        <v>109</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -3657,6 +3684,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H77" t="n">
+        <v>109</v>
+      </c>
+      <c r="I77" t="n">
+        <v>136</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -3690,6 +3726,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H78" t="n">
+        <v>94</v>
+      </c>
+      <c r="I78" t="n">
+        <v>117</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -3723,6 +3768,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H79" t="n">
+        <v>117</v>
+      </c>
+      <c r="I79" t="n">
+        <v>94</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -3756,6 +3810,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H80" t="n">
+        <v>111</v>
+      </c>
+      <c r="I80" t="n">
+        <v>102</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -3789,6 +3852,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H81" t="n">
+        <v>102</v>
+      </c>
+      <c r="I81" t="n">
+        <v>111</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -3822,6 +3894,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H82" t="n">
+        <v>101</v>
+      </c>
+      <c r="I82" t="n">
+        <v>108</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -3855,6 +3936,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H83" t="n">
+        <v>108</v>
+      </c>
+      <c r="I83" t="n">
+        <v>101</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -3888,6 +3978,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H84" t="n">
+        <v>106</v>
+      </c>
+      <c r="I84" t="n">
+        <v>93</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -3921,6 +4020,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H85" t="n">
+        <v>93</v>
+      </c>
+      <c r="I85" t="n">
+        <v>106</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -3954,6 +4062,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H86" t="n">
+        <v>123</v>
+      </c>
+      <c r="I86" t="n">
+        <v>112</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -3986,6 +4103,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H87" t="n">
+        <v>112</v>
+      </c>
+      <c r="I87" t="n">
+        <v>123</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">

</xml_diff>

<commit_message>
Added NBA Results for Oct 26, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -4146,6 +4146,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H88" t="n">
+        <v>125</v>
+      </c>
+      <c r="I88" t="n">
+        <v>127</v>
+      </c>
+      <c r="J88" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -4179,6 +4188,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H89" t="n">
+        <v>127</v>
+      </c>
+      <c r="I89" t="n">
+        <v>125</v>
+      </c>
+      <c r="J89" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -4212,6 +4230,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H90" t="n">
+        <v>103</v>
+      </c>
+      <c r="I90" t="n">
+        <v>110</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -4245,6 +4272,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H91" t="n">
+        <v>110</v>
+      </c>
+      <c r="I91" t="n">
+        <v>103</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -4278,6 +4314,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H92" t="n">
+        <v>113</v>
+      </c>
+      <c r="I92" t="n">
+        <v>109</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -4311,6 +4356,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H93" t="n">
+        <v>109</v>
+      </c>
+      <c r="I93" t="n">
+        <v>113</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -4344,6 +4398,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H94" t="n">
+        <v>99</v>
+      </c>
+      <c r="I94" t="n">
+        <v>134</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -4377,6 +4440,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H95" t="n">
+        <v>134</v>
+      </c>
+      <c r="I95" t="n">
+        <v>99</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -4410,6 +4482,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H96" t="n">
+        <v>102</v>
+      </c>
+      <c r="I96" t="n">
+        <v>110</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -4443,6 +4524,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H97" t="n">
+        <v>110</v>
+      </c>
+      <c r="I97" t="n">
+        <v>102</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -4476,6 +4566,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H98" t="n">
+        <v>114</v>
+      </c>
+      <c r="I98" t="n">
+        <v>125</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -4509,6 +4608,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H99" t="n">
+        <v>125</v>
+      </c>
+      <c r="I99" t="n">
+        <v>114</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -4542,6 +4650,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H100" t="n">
+        <v>110</v>
+      </c>
+      <c r="I100" t="n">
+        <v>120</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -4575,6 +4692,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H101" t="n">
+        <v>120</v>
+      </c>
+      <c r="I101" t="n">
+        <v>110</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -4608,6 +4734,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H102" t="n">
+        <v>110</v>
+      </c>
+      <c r="I102" t="n">
+        <v>105</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -4641,6 +4776,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H103" t="n">
+        <v>105</v>
+      </c>
+      <c r="I103" t="n">
+        <v>110</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -4674,6 +4818,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H104" t="n">
+        <v>134</v>
+      </c>
+      <c r="I104" t="n">
+        <v>114</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -4706,6 +4859,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H105" t="n">
+        <v>114</v>
+      </c>
+      <c r="I105" t="n">
+        <v>134</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="106">

</xml_diff>

<commit_message>
Added NBA Results for Oct 27, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -4902,6 +4902,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H106" t="n">
+        <v>124</v>
+      </c>
+      <c r="I106" t="n">
+        <v>125</v>
+      </c>
+      <c r="J106" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -4935,6 +4944,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H107" t="n">
+        <v>125</v>
+      </c>
+      <c r="I107" t="n">
+        <v>124</v>
+      </c>
+      <c r="J107" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -4968,6 +4986,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H108" t="n">
+        <v>97</v>
+      </c>
+      <c r="I108" t="n">
+        <v>111</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -5001,6 +5028,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H109" t="n">
+        <v>111</v>
+      </c>
+      <c r="I109" t="n">
+        <v>97</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -5034,6 +5070,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H110" t="n">
+        <v>103</v>
+      </c>
+      <c r="I110" t="n">
+        <v>130</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -5067,6 +5112,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H111" t="n">
+        <v>130</v>
+      </c>
+      <c r="I111" t="n">
+        <v>103</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -5100,6 +5154,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H112" t="n">
+        <v>136</v>
+      </c>
+      <c r="I112" t="n">
+        <v>129</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -5132,6 +5195,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H113" t="n">
+        <v>129</v>
+      </c>
+      <c r="I113" t="n">
+        <v>136</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="114">

</xml_diff>

<commit_message>
Added NBA Results for Oct 28, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -5238,6 +5238,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H114" t="n">
+        <v>129</v>
+      </c>
+      <c r="I114" t="n">
+        <v>117</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -5271,6 +5280,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H115" t="n">
+        <v>117</v>
+      </c>
+      <c r="I115" t="n">
+        <v>129</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -5304,6 +5322,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H116" t="n">
+        <v>111</v>
+      </c>
+      <c r="I116" t="n">
+        <v>121</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -5337,6 +5364,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H117" t="n">
+        <v>121</v>
+      </c>
+      <c r="I117" t="n">
+        <v>111</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -5370,6 +5406,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H118" t="n">
+        <v>114</v>
+      </c>
+      <c r="I118" t="n">
+        <v>109</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -5403,6 +5448,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H119" t="n">
+        <v>109</v>
+      </c>
+      <c r="I119" t="n">
+        <v>114</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -5436,6 +5490,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H120" t="n">
+        <v>89</v>
+      </c>
+      <c r="I120" t="n">
+        <v>97</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -5469,6 +5532,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H121" t="n">
+        <v>97</v>
+      </c>
+      <c r="I121" t="n">
+        <v>89</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -5502,6 +5574,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H122" t="n">
+        <v>99</v>
+      </c>
+      <c r="I122" t="n">
+        <v>129</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -5535,6 +5616,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H123" t="n">
+        <v>129</v>
+      </c>
+      <c r="I123" t="n">
+        <v>99</v>
+      </c>
+      <c r="J123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -5568,6 +5658,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H124" t="n">
+        <v>132</v>
+      </c>
+      <c r="I124" t="n">
+        <v>100</v>
+      </c>
+      <c r="J124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -5601,6 +5700,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H125" t="n">
+        <v>100</v>
+      </c>
+      <c r="I125" t="n">
+        <v>132</v>
+      </c>
+      <c r="J125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -5634,6 +5742,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H126" t="n">
+        <v>119</v>
+      </c>
+      <c r="I126" t="n">
+        <v>114</v>
+      </c>
+      <c r="J126" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -5667,6 +5784,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H127" t="n">
+        <v>114</v>
+      </c>
+      <c r="I127" t="n">
+        <v>119</v>
+      </c>
+      <c r="J127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -5700,6 +5826,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H128" t="n">
+        <v>104</v>
+      </c>
+      <c r="I128" t="n">
+        <v>91</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -5733,6 +5868,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H129" t="n">
+        <v>91</v>
+      </c>
+      <c r="I129" t="n">
+        <v>104</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -5766,6 +5910,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H130" t="n">
+        <v>133</v>
+      </c>
+      <c r="I130" t="n">
+        <v>127</v>
+      </c>
+      <c r="J130" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -5799,6 +5952,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H131" t="n">
+        <v>127</v>
+      </c>
+      <c r="I131" t="n">
+        <v>133</v>
+      </c>
+      <c r="J131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -5832,6 +5994,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H132" t="n">
+        <v>117</v>
+      </c>
+      <c r="I132" t="n">
+        <v>111</v>
+      </c>
+      <c r="J132" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -5865,6 +6036,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H133" t="n">
+        <v>111</v>
+      </c>
+      <c r="I133" t="n">
+        <v>117</v>
+      </c>
+      <c r="J133" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -5898,6 +6078,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H134" t="n">
+        <v>96</v>
+      </c>
+      <c r="I134" t="n">
+        <v>120</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -5931,6 +6120,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H135" t="n">
+        <v>120</v>
+      </c>
+      <c r="I135" t="n">
+        <v>96</v>
+      </c>
+      <c r="J135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -5964,6 +6162,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H136" t="n">
+        <v>103</v>
+      </c>
+      <c r="I136" t="n">
+        <v>87</v>
+      </c>
+      <c r="J136" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -5996,6 +6203,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H137" t="n">
+        <v>87</v>
+      </c>
+      <c r="I137" t="n">
+        <v>103</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="138">

</xml_diff>

<commit_message>
Added NBA Results for Oct 29, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -6246,6 +6246,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H138" t="n">
+        <v>111</v>
+      </c>
+      <c r="I138" t="n">
+        <v>114</v>
+      </c>
+      <c r="J138" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -6279,6 +6288,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H139" t="n">
+        <v>114</v>
+      </c>
+      <c r="I139" t="n">
+        <v>111</v>
+      </c>
+      <c r="J139" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -6312,6 +6330,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H140" t="n">
+        <v>120</v>
+      </c>
+      <c r="I140" t="n">
+        <v>132</v>
+      </c>
+      <c r="J140" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -6345,6 +6372,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H141" t="n">
+        <v>132</v>
+      </c>
+      <c r="I141" t="n">
+        <v>120</v>
+      </c>
+      <c r="J141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -6378,6 +6414,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H142" t="n">
+        <v>124</v>
+      </c>
+      <c r="I142" t="n">
+        <v>103</v>
+      </c>
+      <c r="J142" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -6410,6 +6455,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H143" t="n">
+        <v>103</v>
+      </c>
+      <c r="I143" t="n">
+        <v>124</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="144">

</xml_diff>

<commit_message>
Added NBA Results for Oct 30, 2026
</commit_message>
<xml_diff>
--- a/DBs/nba/Results/NBA_2027_Results.xlsx
+++ b/DBs/nba/Results/NBA_2027_Results.xlsx
@@ -6498,6 +6498,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H144" t="n">
+        <v>79</v>
+      </c>
+      <c r="I144" t="n">
+        <v>95</v>
+      </c>
+      <c r="J144" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -6531,6 +6540,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H145" t="n">
+        <v>95</v>
+      </c>
+      <c r="I145" t="n">
+        <v>79</v>
+      </c>
+      <c r="J145" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -6564,6 +6582,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H146" t="n">
+        <v>111</v>
+      </c>
+      <c r="I146" t="n">
+        <v>125</v>
+      </c>
+      <c r="J146" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -6597,6 +6624,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H147" t="n">
+        <v>125</v>
+      </c>
+      <c r="I147" t="n">
+        <v>111</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -6630,6 +6666,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H148" t="n">
+        <v>110</v>
+      </c>
+      <c r="I148" t="n">
+        <v>94</v>
+      </c>
+      <c r="J148" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -6663,6 +6708,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H149" t="n">
+        <v>94</v>
+      </c>
+      <c r="I149" t="n">
+        <v>110</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -6696,6 +6750,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H150" t="n">
+        <v>93</v>
+      </c>
+      <c r="I150" t="n">
+        <v>98</v>
+      </c>
+      <c r="J150" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -6729,6 +6792,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H151" t="n">
+        <v>98</v>
+      </c>
+      <c r="I151" t="n">
+        <v>93</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -6762,6 +6834,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H152" t="n">
+        <v>121</v>
+      </c>
+      <c r="I152" t="n">
+        <v>114</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -6795,6 +6876,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H153" t="n">
+        <v>114</v>
+      </c>
+      <c r="I153" t="n">
+        <v>121</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -6828,6 +6918,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H154" t="n">
+        <v>111</v>
+      </c>
+      <c r="I154" t="n">
+        <v>116</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -6861,6 +6960,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H155" t="n">
+        <v>116</v>
+      </c>
+      <c r="I155" t="n">
+        <v>111</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -6894,6 +7002,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H156" t="n">
+        <v>125</v>
+      </c>
+      <c r="I156" t="n">
+        <v>145</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -6927,6 +7044,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H157" t="n">
+        <v>145</v>
+      </c>
+      <c r="I157" t="n">
+        <v>125</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -6960,6 +7086,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H158" t="n">
+        <v>101</v>
+      </c>
+      <c r="I158" t="n">
+        <v>127</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -6993,6 +7128,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H159" t="n">
+        <v>127</v>
+      </c>
+      <c r="I159" t="n">
+        <v>101</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -7026,6 +7170,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H160" t="n">
+        <v>95</v>
+      </c>
+      <c r="I160" t="n">
+        <v>112</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -7059,6 +7212,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H161" t="n">
+        <v>112</v>
+      </c>
+      <c r="I161" t="n">
+        <v>95</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -7092,6 +7254,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H162" t="n">
+        <v>127</v>
+      </c>
+      <c r="I162" t="n">
+        <v>120</v>
+      </c>
+      <c r="J162" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -7124,6 +7295,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H163" t="n">
+        <v>120</v>
+      </c>
+      <c r="I163" t="n">
+        <v>127</v>
+      </c>
+      <c r="J163" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="164">

</xml_diff>